<commit_message>
test(compressor_v2): use block_size param for state_cache, register cpv2.compressor op
- pt_save/golden: build state_cache with passed-in block_size, drop min-1024 cap
- compressor.py: register torch.ops op as cann_ops_transformer::cpv2.compressor
- excel: add S8K_B128 case (S=8k, block_size=128)
</commit_message>
<xml_diff>
--- a/experimental/attention/compressor_v2/tests/pytest/excel/test_cases.xlsx
+++ b/experimental/attention/compressor_v2/tests/pytest/excel/test_cases.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2104,6 +2104,76 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>S8K_B128</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>4096</v>
+      </c>
+      <c r="D26" t="n">
+        <v>8192</v>
+      </c>
+      <c r="E26" t="n">
+        <v>512</v>
+      </c>
+      <c r="F26" t="n">
+        <v>128</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>BF16</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>0,8192</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>-3,3</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>-5,5</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>-5,5</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>-10,10</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>-10,10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(compressor_v2): add is_contiguous switch for state_cache and fix batch golden
The operator is fixed to cache_mode=2 (ring buffer). Unify the state_cache
construction in golden/loadprocess to build the padded view on NPU (pad moved
to NPU before creating the non-contiguous view), previously the view stayed on
CPU causing device errors.

Add an optional is_contiguous switch (default false = non-contiguous):
- single test: run_compressor_eager(is_contiguous=...) + Contiguous0 /
  NonContiguous0 cases in the full case list
- batch test: optional is_contiguous excel column threaded through pt_save into
  pt_loadprocess; document it in BATCH_GUIDE.md

Verified: single and batch both pass for contiguous (pad=0) and non-contiguous
(pad>0) state_cache.
</commit_message>
<xml_diff>
--- a/experimental/attention/compressor_v2/tests/pytest/excel/test_cases.xlsx
+++ b/experimental/attention/compressor_v2/tests/pytest/excel/test_cases.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,11 @@
           <t>score_state_datarange</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>is_contiguous</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -585,6 +590,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -651,6 +659,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -717,6 +728,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -783,6 +797,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -849,6 +866,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -915,6 +935,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -981,6 +1004,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1047,6 +1073,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1113,6 +1142,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1179,6 +1211,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1245,6 +1280,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1311,6 +1349,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1377,6 +1418,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1443,6 +1487,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1509,6 +1556,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1575,6 +1625,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1641,6 +1694,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1707,6 +1763,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1773,6 +1832,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1839,6 +1901,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1905,6 +1970,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1971,6 +2039,9 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2037,21 +2108,24 @@
           <t>-10,10</t>
         </is>
       </c>
+      <c r="S24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MyRandomCase</t>
+          <t>Contiguous0</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
         <v>4096</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
         <v>512</v>
@@ -2063,11 +2137,11 @@
         <v>4</v>
       </c>
       <c r="H25" t="n">
-        <v>100</v>
+        <v>8193</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BSH</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2080,17 +2154,17 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>-3,3</t>
+          <t>-10,10</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>-5,5</t>
+          <t>-10,10</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>-5,5</t>
+          <t>-10,10</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2102,22 +2176,25 @@
         <is>
           <t>-10,10</t>
         </is>
+      </c>
+      <c r="S25" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>S8K_B128</t>
+          <t>NonContiguous0</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="n">
         <v>4096</v>
       </c>
       <c r="D26" t="n">
-        <v>8192</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
         <v>512</v>
@@ -2129,7 +2206,7 @@
         <v>4</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>8193</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2141,26 +2218,22 @@
           <t>BF16</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>0,8192</t>
-        </is>
-      </c>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>-3,3</t>
+          <t>-10,10</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>-5,5</t>
+          <t>-10,10</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>-5,5</t>
+          <t>-10,10</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -2172,6 +2245,9 @@
         <is>
           <t>-10,10</t>
         </is>
+      </c>
+      <c r="S26" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>